<commit_message>
Enhance data processing scripts for poverty and employment analysis
- Updated Stata scripts to improve variable handling and dataset management.
- Added logic to dynamically include relevant survey variables based on year.
- Cleaned up unnecessary code and improved readability in the employment dashboard script.
- Removed temporary Excel files that are no longer needed.
</commit_message>
<xml_diff>
--- a/Dashboards/data/Data final/empleo/empleo adecuado/empleo_series.xlsx
+++ b/Dashboards/data/Data final/empleo/empleo adecuado/empleo_series.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <workbookPr/>
   <bookViews>
     <workbookView activeTab="0"/>
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="60" uniqueCount="6">
   <si>
     <t>anio</t>
   </si>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -75,7 +75,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C58"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -362,7 +362,7 @@
         <v>2</v>
       </c>
       <c r="C26" s="1">
-        <v>4.7728347778320312</v>
+        <v>4.7728347778320313</v>
       </c>
     </row>
     <row r="27">

</xml_diff>